<commit_message>
Cabmio de archivo, se subió la plantilla vacía.
</commit_message>
<xml_diff>
--- a/Documentacion/FuncionalidadesSignificativas.xlsx
+++ b/Documentacion/FuncionalidadesSignificativas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wsancheg\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/F3F179366C32E272/Documentos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{836D7EDD-CE4D-46C4-AED5-090A68C0CC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AFE37B1-284C-418B-A105-DC2C0B35F298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{49B2EC2E-3F64-4369-B5EE-BCFE592BC9C3}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" firstSheet="1" activeTab="1" xr2:uid="{49B2EC2E-3F64-4369-B5EE-BCFE592BC9C3}"/>
   </bookViews>
   <sheets>
     <sheet name="HU" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="210">
   <si>
     <t>Nombre Historia de Usuario</t>
   </si>
@@ -511,23 +511,170 @@
     <t>Observación</t>
   </si>
   <si>
+    <t>RF-001</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir al supervisor de campo registrar la siembra de una cama (bloque, nave, cama, variedad, fecha y cantidad de esquejes) sin conexion a internet, confirmando en pantalla que el registro quedo guardado en el dispositivo.</t>
+  </si>
+  <si>
+    <t>Valor de negocio</t>
+  </si>
+  <si>
+    <t>Es una parte principal del funcionamiento esperado del producto, sin esta información se haría imposible realizar la proyección de datos que el cliente espera tener disponible en cualquier momento, sin esta funcionalidad no habría información sobre la cual el resto del producto pueda funcionar correctamente.</t>
+  </si>
+  <si>
+    <t>RF-002</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir al supervisor de campo registrar el corte de una cama por variedad, grado y fecha sin conexion a internet, aceptando varios registros de corte para la misma cama en dias distintos de su ciclo.</t>
+  </si>
+  <si>
+    <t>RF-003</t>
+  </si>
+  <si>
+    <t>El sistema debe sincronizar los registros capturados en el dispositivo con el repositorio central cuando haya conectividad, garantizando que ningun registro se pierda y que ninguno se aplique mas de una vez.</t>
+  </si>
+  <si>
+    <t>Ambos</t>
+  </si>
+  <si>
+    <t>El cliente cuenta con una forma con la cual pueda verificar información de manera rápida para realizar correcciones de la toma de datos realizada en el campo dónde no se cuenta con conexión para mantener un seguimiento constante de esta información, dando así la necesidad de abordar esta sincronización cómo reto técnico y valor de negocio debido a su importancia en el proceso de analisis de datos que el cliente necesita realizar.</t>
+  </si>
+  <si>
+    <t>RF-004</t>
+  </si>
+  <si>
+    <t>El sistema debe impedir el registro de un evento que sea imposible dentro del ciclo fenologico de la cama y explicar al usuario el motivo del rechazo, aun sin conexion a internet.</t>
+  </si>
+  <si>
+    <t>Es necesario ofrecer una forma de avisar al usuario cuando un registro inclumple las reglas del negocio de manera offline, esto para poder asegurar la calidad de los datos antes de realizar un proceso de sincronización. Hoy el proceso tiene un porcentaje de error de recolecta de datos del 2% debido a la imposbilidad de verificar información de manera inmediata.</t>
+  </si>
+  <si>
+    <t>RF-005</t>
+  </si>
+  <si>
+    <t>El sistema debe rechazar todo dato de produccion que implique una cantidad de tallos superior a la cantidad de plantas sembradas en esa cama.</t>
+  </si>
+  <si>
+    <t>Debido al funcionamiento del negocio dónde el registro se indica cómo una cantidad definida por superficie definida es importante para el correcto funcionamiento del negocio que se pueda evitar problemas de recolección de datos de manera inmediata.</t>
+  </si>
+  <si>
+    <t>RF-006</t>
+  </si>
+  <si>
+    <t>El sistema debe calcular los tallos proyectados de una cama a partir de su area, de la densidad de siembra definida para la variedad y del porcentaje de productividad esperada de esa variedad.</t>
+  </si>
+  <si>
+    <t>Es importante para la plataforma resaltar y definir de manera pronta el funcionamiento de la estimación de tallos que se aplica dentro del negocio para su uso dentro de la proyección de producción, sin esta funcionalidad los datos capturados no se adaptarían a los modelos utilizados actualmente dentro de las empresas.</t>
+  </si>
+  <si>
+    <t>Los tallos son la forma en la que se conoce dentro del negocio a 1 planta, esta planta cuenta con diferentes caracteristicas</t>
+  </si>
+  <si>
+    <t>RF-008</t>
+  </si>
+  <si>
+    <t>El sistema debe regenerar la proyeccion con la informacion acumulada al menos una vez por semana conservando la version anterior de cada proyeccion generada.</t>
+  </si>
+  <si>
+    <t>Este es un punto crítico que busca al cliente ahorrar el tiempo cómo fue solicitado por él mismo, el proceso actual sin plataforma puede demorarse 1 mes, para realizar la proyección de producción.</t>
+  </si>
+  <si>
+    <t>La proyección que es necesaria para definir los recursos con los que se pueden contar a la hora de realizar ventas</t>
+  </si>
+  <si>
+    <t>RF-009</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir registrar la erradicacion parcial o total de una cama descontando esta información en procesos proximos de la captura de datos modificando la produccion que quedaba proyectada para esa cama.</t>
+  </si>
+  <si>
+    <t>Normalmente no se espera que la producción de una cama siempre salga cómo lo esperado, por lo que por diferentes causas o factores dentro del proceso de producción puede haber una reducción de producto dentro de la cama, esta información afecta directmante a la proyección que busca el cliente.</t>
+  </si>
+  <si>
+    <t>RF-011</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar la desviacion entre el corte real y el corte proyectado por cama, variedad y periodo, senalando los casos que salen de la banda de tolerancia parametrizada.</t>
+  </si>
+  <si>
+    <t>Es la forma en la que le puedo garantizar al cliente que el uso de la flataforma mejora sus métricas ofreciendo más precisión que los métodos anteriores a los cuales estaba acostumbrado, es una forma en la que se le da valor al negocio con un aspecto medible para el usuario final.</t>
+  </si>
+  <si>
+    <t>RF-012</t>
+  </si>
+  <si>
+    <t>El sistema debe garantizar que ningun usuario pueda acceder, por ningun canal, a datos pertenecientes a una empresa distinta de aquella a la que pertenece su cuenta.</t>
+  </si>
+  <si>
+    <t>A peticion del cliente es necesario que cada empresa tenga la seguridad de que ninguno de sus datos puedan ser visualizados por personas ajenas a ellos devido a la importancia que hay en sus datos</t>
+  </si>
+  <si>
+    <t>RF-013</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir al administrador de cada empresa parametrizar sus variedades, densidades de siembra, porcentajes de productividad esperada, grados de calidad, dias a corte por etapa, duracion del corte y bandas de tolerancia, sin intervencion del equipo de desarrollo.</t>
+  </si>
+  <si>
+    <t>Debido al enfoque SaaS que se quiere adoptar para el negocio, es necesario poder contar con las facilidades de personalización indicadas para poder empezar el proceso de captura de datos y proyección.</t>
+  </si>
+  <si>
+    <t>RF-014</t>
+  </si>
+  <si>
+    <t>El sistema debe autenticar al usuario y aplicar los permisos de su rol en el dispositivo movil aun cuando no haya conexion a internet.</t>
+  </si>
+  <si>
+    <t>Es necesario poder ofrecerle al cliente final la forma de poder identificar la persona que realizó la captura de datos para poder dar seguimiento a la información y cómo esta es ingresada, en entornos que no cuenten con acceso a internet.</t>
+  </si>
+  <si>
+    <t>RF-016</t>
+  </si>
+  <si>
+    <t>El sistema debe conservar, para cada registro de siembra, corte, baja y erradicacion, la empresa, el autor, el dispositivo, la fecha y hora de captura, la fecha de sincronizacion y el valor anterior en caso de correccion.</t>
+  </si>
+  <si>
+    <t>El usuario final tiene un porcentaje de error que dificulta o empeora su proceso de ventas, para evitarlo es necesario que la plataforma pueda identificar quien, cómo, cuándo y evitar la entrada de información erronea que pueda comprometer los datos de sus proyecciónes.</t>
+  </si>
+  <si>
+    <t>RF-017</t>
+  </si>
+  <si>
+    <t>El sistema debe impedir que un registro ya sincronizado sea modificado o eliminado por un rol distinto del administrador de la empresa, y debe exigir que quede registrada la aprobacion que respalda la correccion.</t>
+  </si>
+  <si>
+    <t>Para mantener la trazabilidad y la integridad de los datos es necesario que solo el rol de administrador de produccion tenga la capacidad para hacer cambios o eliminar los datos, manteniendo asi la confianza total sobre los datos capturados</t>
+  </si>
+  <si>
+    <t>RF-018</t>
+  </si>
+  <si>
+    <t>El sistema debe presentar la produccion proyectada y la produccion real agregadas por dia, por semana y por mes, calculadas sobre el mismo conjunto de datos.</t>
+  </si>
+  <si>
+    <t>Para la empresa es muy importante poder visualizar esta diferencia para la toma de desiciones, pero esta informacion la ven de forma diferente dependiendo del rol dentro de la empresa, la gerencia general lo busca mensual, el gerente de ventas semanal y el de produccion diario.</t>
+  </si>
+  <si>
+    <t>RF-019</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir exportar a Excel y a PDF la informacion que el usuario tiene autorizado consultar, aplicando las mismas restricciones de rol que rigen en pantalla.</t>
+  </si>
+  <si>
+    <t>Debido a la gran variedad de tipos de usuario que puede presentar una empresa se definió realizar una forma de compartir información adaptada a lo que el negocio más utiliza ahorrandole así la necesidad de una gestión de roles pesada.</t>
+  </si>
+  <si>
     <t>Tipo funcionalidad significativa</t>
   </si>
   <si>
-    <t>Valor de negocio</t>
-  </si>
-  <si>
     <t>Reto técnico</t>
-  </si>
-  <si>
-    <t>Ambos</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -554,6 +701,17 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -619,7 +777,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -640,26 +798,38 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -976,7 +1146,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3E6C96F-D3DF-42C6-B304-FF994E2AF637}">
   <dimension ref="A1:B76"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="28.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.42578125" style="1" customWidth="1"/>
@@ -990,7 +1160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="72.599999999999994">
+    <row r="2" spans="1:2" ht="57">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -998,7 +1168,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="57.95">
+    <row r="3" spans="1:2" ht="57">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1006,7 +1176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="57.95">
+    <row r="4" spans="1:2" ht="57">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1014,7 +1184,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="87">
+    <row r="5" spans="1:2" ht="85.5">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
@@ -1022,7 +1192,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="72.599999999999994">
+    <row r="6" spans="1:2" ht="71.25">
       <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
@@ -1030,7 +1200,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="87">
+    <row r="7" spans="1:2" ht="71.25">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
@@ -1038,7 +1208,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="43.5">
+    <row r="8" spans="1:2" ht="42.75">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
@@ -1046,7 +1216,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="57.95">
+    <row r="9" spans="1:2" ht="57">
       <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
@@ -1054,7 +1224,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="57.95">
+    <row r="10" spans="1:2" ht="57">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -1062,7 +1232,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="72.599999999999994">
+    <row r="11" spans="1:2" ht="57">
       <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
@@ -1070,7 +1240,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="57.95">
+    <row r="12" spans="1:2" ht="57">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -1078,7 +1248,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="72.599999999999994">
+    <row r="13" spans="1:2" ht="57">
       <c r="A13" s="3" t="s">
         <v>24</v>
       </c>
@@ -1086,7 +1256,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="57.95">
+    <row r="14" spans="1:2" ht="57">
       <c r="A14" s="3" t="s">
         <v>26</v>
       </c>
@@ -1094,7 +1264,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="43.5">
+    <row r="15" spans="1:2" ht="42.75">
       <c r="A15" s="3" t="s">
         <v>28</v>
       </c>
@@ -1102,7 +1272,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="57.95">
+    <row r="16" spans="1:2" ht="57">
       <c r="A16" s="3" t="s">
         <v>30</v>
       </c>
@@ -1110,7 +1280,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="72.599999999999994">
+    <row r="17" spans="1:2" ht="57">
       <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
@@ -1118,7 +1288,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="57.95">
+    <row r="18" spans="1:2" ht="57">
       <c r="A18" s="3" t="s">
         <v>34</v>
       </c>
@@ -1126,7 +1296,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="57.95">
+    <row r="19" spans="1:2" ht="57">
       <c r="A19" s="3" t="s">
         <v>36</v>
       </c>
@@ -1134,7 +1304,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="87">
+    <row r="20" spans="1:2" ht="85.5">
       <c r="A20" s="3" t="s">
         <v>38</v>
       </c>
@@ -1142,7 +1312,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="72.599999999999994">
+    <row r="21" spans="1:2" ht="57">
       <c r="A21" s="3" t="s">
         <v>40</v>
       </c>
@@ -1150,7 +1320,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="87">
+    <row r="22" spans="1:2" ht="71.25">
       <c r="A22" s="3" t="s">
         <v>42</v>
       </c>
@@ -1158,7 +1328,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="72.599999999999994">
+    <row r="23" spans="1:2" ht="57">
       <c r="A23" s="3" t="s">
         <v>44</v>
       </c>
@@ -1166,7 +1336,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="87">
+    <row r="24" spans="1:2" ht="85.5">
       <c r="A24" s="3" t="s">
         <v>46</v>
       </c>
@@ -1174,7 +1344,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="72.599999999999994">
+    <row r="25" spans="1:2" ht="71.25">
       <c r="A25" s="3" t="s">
         <v>48</v>
       </c>
@@ -1182,7 +1352,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="87">
+    <row r="26" spans="1:2" ht="71.25">
       <c r="A26" s="3" t="s">
         <v>50</v>
       </c>
@@ -1190,7 +1360,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="72.599999999999994">
+    <row r="27" spans="1:2" ht="57">
       <c r="A27" s="3" t="s">
         <v>52</v>
       </c>
@@ -1198,7 +1368,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="57.95">
+    <row r="28" spans="1:2" ht="57">
       <c r="A28" s="3" t="s">
         <v>54</v>
       </c>
@@ -1206,7 +1376,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="72.599999999999994">
+    <row r="29" spans="1:2" ht="57">
       <c r="A29" s="3" t="s">
         <v>56</v>
       </c>
@@ -1214,7 +1384,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="57.95">
+    <row r="30" spans="1:2" ht="57">
       <c r="A30" s="3" t="s">
         <v>58</v>
       </c>
@@ -1222,7 +1392,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="57.95">
+    <row r="31" spans="1:2" ht="57">
       <c r="A31" s="3" t="s">
         <v>60</v>
       </c>
@@ -1230,7 +1400,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="57.95">
+    <row r="32" spans="1:2" ht="57">
       <c r="A32" s="3" t="s">
         <v>62</v>
       </c>
@@ -1238,7 +1408,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="72.599999999999994">
+    <row r="33" spans="1:2" ht="57">
       <c r="A33" s="3" t="s">
         <v>64</v>
       </c>
@@ -1246,7 +1416,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="57.95">
+    <row r="34" spans="1:2" ht="57">
       <c r="A34" s="3" t="s">
         <v>66</v>
       </c>
@@ -1254,7 +1424,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="72.599999999999994">
+    <row r="35" spans="1:2" ht="57">
       <c r="A35" s="3" t="s">
         <v>68</v>
       </c>
@@ -1262,7 +1432,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="57.95">
+    <row r="36" spans="1:2" ht="57">
       <c r="A36" s="3" t="s">
         <v>70</v>
       </c>
@@ -1270,7 +1440,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="57.95">
+    <row r="37" spans="1:2" ht="57">
       <c r="A37" s="3" t="s">
         <v>72</v>
       </c>
@@ -1278,7 +1448,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="72.599999999999994">
+    <row r="38" spans="1:2" ht="71.25">
       <c r="A38" s="3" t="s">
         <v>74</v>
       </c>
@@ -1286,7 +1456,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="57.95">
+    <row r="39" spans="1:2" ht="57">
       <c r="A39" s="3" t="s">
         <v>76</v>
       </c>
@@ -1294,7 +1464,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="57.95">
+    <row r="40" spans="1:2" ht="57">
       <c r="A40" s="3" t="s">
         <v>78</v>
       </c>
@@ -1302,7 +1472,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="57.95">
+    <row r="41" spans="1:2" ht="57">
       <c r="A41" s="3" t="s">
         <v>80</v>
       </c>
@@ -1310,7 +1480,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="72.599999999999994">
+    <row r="42" spans="1:2" ht="57">
       <c r="A42" s="3" t="s">
         <v>82</v>
       </c>
@@ -1318,7 +1488,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="57.95">
+    <row r="43" spans="1:2" ht="57">
       <c r="A43" s="3" t="s">
         <v>84</v>
       </c>
@@ -1326,7 +1496,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="57.95">
+    <row r="44" spans="1:2" ht="57">
       <c r="A44" s="3" t="s">
         <v>86</v>
       </c>
@@ -1334,7 +1504,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="43.5">
+    <row r="45" spans="1:2" ht="42.75">
       <c r="A45" s="3" t="s">
         <v>88</v>
       </c>
@@ -1342,7 +1512,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="57.95">
+    <row r="46" spans="1:2" ht="57">
       <c r="A46" s="3" t="s">
         <v>90</v>
       </c>
@@ -1350,7 +1520,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="43.5">
+    <row r="47" spans="1:2" ht="42.75">
       <c r="A47" s="3" t="s">
         <v>92</v>
       </c>
@@ -1358,7 +1528,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="72.599999999999994">
+    <row r="48" spans="1:2" ht="57">
       <c r="A48" s="3" t="s">
         <v>94</v>
       </c>
@@ -1366,7 +1536,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="43.5">
+    <row r="49" spans="1:2" ht="42.75">
       <c r="A49" s="3" t="s">
         <v>96</v>
       </c>
@@ -1374,7 +1544,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="87">
+    <row r="50" spans="1:2" ht="85.5">
       <c r="A50" s="3" t="s">
         <v>98</v>
       </c>
@@ -1382,7 +1552,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="57.95">
+    <row r="51" spans="1:2" ht="57">
       <c r="A51" s="3" t="s">
         <v>100</v>
       </c>
@@ -1390,7 +1560,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="72.599999999999994">
+    <row r="52" spans="1:2" ht="71.25">
       <c r="A52" s="3" t="s">
         <v>102</v>
       </c>
@@ -1398,7 +1568,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="87">
+    <row r="53" spans="1:2" ht="71.25">
       <c r="A53" s="3" t="s">
         <v>104</v>
       </c>
@@ -1406,7 +1576,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="72.599999999999994">
+    <row r="54" spans="1:2" ht="57">
       <c r="A54" s="3" t="s">
         <v>106</v>
       </c>
@@ -1414,7 +1584,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="72.599999999999994">
+    <row r="55" spans="1:2" ht="57">
       <c r="A55" s="3" t="s">
         <v>108</v>
       </c>
@@ -1422,7 +1592,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="72.599999999999994">
+    <row r="56" spans="1:2" ht="57">
       <c r="A56" s="3" t="s">
         <v>110</v>
       </c>
@@ -1430,7 +1600,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="72.599999999999994">
+    <row r="57" spans="1:2" ht="71.25">
       <c r="A57" s="3" t="s">
         <v>112</v>
       </c>
@@ -1438,7 +1608,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="72.599999999999994">
+    <row r="58" spans="1:2" ht="71.25">
       <c r="A58" s="3" t="s">
         <v>114</v>
       </c>
@@ -1446,7 +1616,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="87">
+    <row r="59" spans="1:2" ht="85.5">
       <c r="A59" s="3" t="s">
         <v>116</v>
       </c>
@@ -1454,7 +1624,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="57.95">
+    <row r="60" spans="1:2" ht="57">
       <c r="A60" s="3" t="s">
         <v>118</v>
       </c>
@@ -1462,7 +1632,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="72.599999999999994">
+    <row r="61" spans="1:2" ht="57">
       <c r="A61" s="3" t="s">
         <v>120</v>
       </c>
@@ -1470,7 +1640,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="57.95">
+    <row r="62" spans="1:2" ht="42.75">
       <c r="A62" s="3" t="s">
         <v>122</v>
       </c>
@@ -1478,7 +1648,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="43.5">
+    <row r="63" spans="1:2" ht="42.75">
       <c r="A63" s="3" t="s">
         <v>124</v>
       </c>
@@ -1486,7 +1656,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="43.5">
+    <row r="64" spans="1:2" ht="42.75">
       <c r="A64" s="3" t="s">
         <v>126</v>
       </c>
@@ -1494,7 +1664,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="72.599999999999994">
+    <row r="65" spans="1:2" ht="57">
       <c r="A65" s="3" t="s">
         <v>128</v>
       </c>
@@ -1502,7 +1672,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="72.599999999999994">
+    <row r="66" spans="1:2" ht="57">
       <c r="A66" s="3" t="s">
         <v>130</v>
       </c>
@@ -1510,7 +1680,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="72.599999999999994">
+    <row r="67" spans="1:2" ht="57">
       <c r="A67" s="3" t="s">
         <v>132</v>
       </c>
@@ -1518,7 +1688,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="72.599999999999994">
+    <row r="68" spans="1:2" ht="71.25">
       <c r="A68" s="3" t="s">
         <v>134</v>
       </c>
@@ -1526,7 +1696,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="72.599999999999994">
+    <row r="69" spans="1:2" ht="71.25">
       <c r="A69" s="3" t="s">
         <v>136</v>
       </c>
@@ -1534,7 +1704,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="72.599999999999994">
+    <row r="70" spans="1:2" ht="57">
       <c r="A70" s="3" t="s">
         <v>138</v>
       </c>
@@ -1542,7 +1712,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="72.599999999999994">
+    <row r="71" spans="1:2" ht="57">
       <c r="A71" s="3" t="s">
         <v>140</v>
       </c>
@@ -1550,7 +1720,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="72.599999999999994">
+    <row r="72" spans="1:2" ht="57">
       <c r="A72" s="3" t="s">
         <v>142</v>
       </c>
@@ -1558,7 +1728,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="72.599999999999994">
+    <row r="73" spans="1:2" ht="57">
       <c r="A73" s="3" t="s">
         <v>144</v>
       </c>
@@ -1574,7 +1744,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="72.599999999999994">
+    <row r="75" spans="1:2" ht="71.25">
       <c r="A75" s="3" t="s">
         <v>148</v>
       </c>
@@ -1582,7 +1752,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="72.599999999999994">
+    <row r="76" spans="1:2" ht="71.25">
       <c r="A76" s="3" t="s">
         <v>150</v>
       </c>
@@ -1597,63 +1767,280 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9CBA1D8-18C8-4CD8-9CD7-BD7764D97086}">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.45"/>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="4" customWidth="1"/>
-    <col min="2" max="3" width="32.42578125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="56" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.42578125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="58" style="5" customWidth="1"/>
     <col min="5" max="5" width="48.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="10.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="43.5">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:5" ht="42.75">
+      <c r="A1" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="11" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="13"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="14"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="13"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="14"/>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="13"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="13"/>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
+    <row r="2" spans="1:5" ht="69" customHeight="1">
+      <c r="A2" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="E2" s="7"/>
+    </row>
+    <row r="3" spans="1:5" ht="69" customHeight="1">
+      <c r="A3" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="18"/>
+      <c r="E3" s="7"/>
+    </row>
+    <row r="4" spans="1:5" ht="107.25" customHeight="1">
+      <c r="A4" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" s="14"/>
+    </row>
+    <row r="5" spans="1:5" ht="115.5" customHeight="1">
+      <c r="A5" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E5" s="7"/>
+    </row>
+    <row r="6" spans="1:5" ht="75" customHeight="1">
+      <c r="A6" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="E6" s="7"/>
+    </row>
+    <row r="7" spans="1:5" ht="87" customHeight="1">
+      <c r="A7" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="95.25" customHeight="1">
+      <c r="A8" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="75.75" customHeight="1">
+      <c r="A9" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="E9" s="7"/>
+    </row>
+    <row r="10" spans="1:5" ht="81" customHeight="1">
+      <c r="A10" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" spans="1:5" ht="55.5" customHeight="1">
+      <c r="A11" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="E11" s="7"/>
+    </row>
+    <row r="12" spans="1:5" ht="64.150000000000006">
+      <c r="A12" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="E12" s="7"/>
+    </row>
+    <row r="13" spans="1:5" ht="84" customHeight="1">
+      <c r="A13" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:5" ht="84.75" customHeight="1">
+      <c r="A14" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="E14" s="7"/>
+    </row>
+    <row r="15" spans="1:5" ht="76.5" customHeight="1">
+      <c r="A15" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="E15" s="7"/>
+    </row>
+    <row r="16" spans="1:5" ht="55.5" customHeight="1">
+      <c r="A16" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="E16" s="7"/>
+    </row>
+    <row r="17" spans="1:5" ht="78" customHeight="1">
+      <c r="A17" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="E17" s="7"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D2:D3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -1662,7 +2049,7 @@
           <x14:formula1>
             <xm:f>Valores!$A$2:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C4</xm:sqref>
+          <xm:sqref>C2:C17</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1673,26 +2060,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{632737A5-F2C7-45B2-B066-A4566BC08B73}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="9" t="s">
-        <v>157</v>
+      <c r="A1" s="8" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>159</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se añadieron requisitos funcionales críticos importantes para garantizar la integridad de los datos y la usabilidad de los usuarios.
</commit_message>
<xml_diff>
--- a/Documentacion/FuncionalidadesSignificativas.xlsx
+++ b/Documentacion/FuncionalidadesSignificativas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/F3F179366C32E272/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanp\FlorLogic\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AFE37B1-284C-418B-A105-DC2C0B35F298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B412A36D-97C7-4F5D-A88F-51AA4D21F67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" firstSheet="1" activeTab="1" xr2:uid="{49B2EC2E-3F64-4369-B5EE-BCFE592BC9C3}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{49B2EC2E-3F64-4369-B5EE-BCFE592BC9C3}"/>
   </bookViews>
   <sheets>
     <sheet name="HU" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="226">
   <si>
     <t>Nombre Historia de Usuario</t>
   </si>
@@ -668,13 +668,61 @@
   </si>
   <si>
     <t>Reto técnico</t>
+  </si>
+  <si>
+    <t>RF-020</t>
+  </si>
+  <si>
+    <t>El sistema de exigir y garantizar la descarga de la parametrización más reciente con la información relevante para permitir la captura de datos (cómo: Variedades, camas, reglas de negocio) en el dispositivo.</t>
+  </si>
+  <si>
+    <t>Sin esta información el supervisor de campo no podría registrar el algún cambio en una cama o lo haría en una cama inexistente.</t>
+  </si>
+  <si>
+    <t>RF-021</t>
+  </si>
+  <si>
+    <t>El sistema debe registrar una marca en el tiempo inmutable en cada evento capturado de manera offline, bloqueando el registro si se detecta alteración manual en el reloj del dispositivo.</t>
+  </si>
+  <si>
+    <t>Los ciclos fenológicos de los tallos sobre los cuales se estima la proyección son sensibles a desfases en el tiempo en sus actividades, es necesario llevar registro real de tiempo.</t>
+  </si>
+  <si>
+    <t>Los ciclos fenológicos son los cambios en las etapas de crecimiento de los cultivos de flores.</t>
+  </si>
+  <si>
+    <t>RF-022</t>
+  </si>
+  <si>
+    <t>Se pueden dar casos dónde diferentes supervisores recolecten información en plazos muy cortos de tiempo y sobre la misma cama, es indispensable poder llevar un seguimiento de los cambios si se da el caso que se modifique la misma información por dos fuentes distinas.</t>
+  </si>
+  <si>
+    <t>FR-023</t>
+  </si>
+  <si>
+    <t>El sistema debe realizar una captura estática en el tiempo sobre los parámetros de calculo y proyección permitiendo ignorar cambios que puedan reducir la consistencia de los datos.</t>
+  </si>
+  <si>
+    <t>Es necesario ofrecer al usuario una forma de gestión de versionamiento para poder asegurar que la información determinada cómo estable o adecuada por los usuarios no sea corrompida por un cambio simple en etapas adelantas del ciclo fenológico.</t>
+  </si>
+  <si>
+    <t>El sistema debe identifica e informar de manera visual y clara la causa de una caída en la producción proyectada especificando el motivo de la caída.</t>
+  </si>
+  <si>
+    <t>El usuario solocitó mostrar la información para predecir. Si el sistema cambia la proyección esperada sin explicar el motivo, el usuario no podría tomar acciones al respecto.</t>
+  </si>
+  <si>
+    <t>FR-024</t>
+  </si>
+  <si>
+    <t>El sistema debe resolver conflictos de información sincronizada en el sistema, aplicando un orden cronológico estricto permitiendo a los administradores consultar un registro de cambios.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -713,6 +761,14 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -819,17 +875,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -849,9 +905,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -889,7 +945,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -995,7 +1051,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1137,7 +1193,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1146,13 +1202,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3E6C96F-D3DF-42C6-B304-FF994E2AF637}">
   <dimension ref="A1:B76"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="46.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="28.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="46.44140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1160,7 +1216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="57">
+    <row r="2" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1168,7 +1224,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="57">
+    <row r="3" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1176,7 +1232,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="57">
+    <row r="4" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1184,7 +1240,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="85.5">
+    <row r="5" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
@@ -1192,7 +1248,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="71.25">
+    <row r="6" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
@@ -1200,7 +1256,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="71.25">
+    <row r="7" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
@@ -1208,7 +1264,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="42.75">
+    <row r="8" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
@@ -1216,7 +1272,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="57">
+    <row r="9" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
@@ -1224,7 +1280,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="57">
+    <row r="10" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -1232,7 +1288,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="57">
+    <row r="11" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
@@ -1240,7 +1296,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="57">
+    <row r="12" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -1248,7 +1304,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="57">
+    <row r="13" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>24</v>
       </c>
@@ -1256,7 +1312,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="57">
+    <row r="14" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>26</v>
       </c>
@@ -1264,7 +1320,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="42.75">
+    <row r="15" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>28</v>
       </c>
@@ -1272,7 +1328,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="57">
+    <row r="16" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>30</v>
       </c>
@@ -1280,7 +1336,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="57">
+    <row r="17" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
@@ -1288,7 +1344,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="57">
+    <row r="18" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>34</v>
       </c>
@@ -1296,7 +1352,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="57">
+    <row r="19" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>36</v>
       </c>
@@ -1304,7 +1360,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="85.5">
+    <row r="20" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>38</v>
       </c>
@@ -1312,7 +1368,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="57">
+    <row r="21" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>40</v>
       </c>
@@ -1320,7 +1376,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="71.25">
+    <row r="22" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>42</v>
       </c>
@@ -1328,7 +1384,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="57">
+    <row r="23" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>44</v>
       </c>
@@ -1336,7 +1392,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="85.5">
+    <row r="24" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>46</v>
       </c>
@@ -1344,7 +1400,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="71.25">
+    <row r="25" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>48</v>
       </c>
@@ -1352,7 +1408,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="71.25">
+    <row r="26" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>50</v>
       </c>
@@ -1360,7 +1416,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="57">
+    <row r="27" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>52</v>
       </c>
@@ -1368,7 +1424,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="57">
+    <row r="28" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>54</v>
       </c>
@@ -1376,7 +1432,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="57">
+    <row r="29" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>56</v>
       </c>
@@ -1384,7 +1440,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="57">
+    <row r="30" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>58</v>
       </c>
@@ -1392,7 +1448,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="57">
+    <row r="31" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>60</v>
       </c>
@@ -1400,7 +1456,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="57">
+    <row r="32" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>62</v>
       </c>
@@ -1408,7 +1464,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="57">
+    <row r="33" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>64</v>
       </c>
@@ -1416,7 +1472,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="57">
+    <row r="34" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>66</v>
       </c>
@@ -1424,7 +1480,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="57">
+    <row r="35" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>68</v>
       </c>
@@ -1432,7 +1488,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="57">
+    <row r="36" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>70</v>
       </c>
@@ -1440,7 +1496,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="57">
+    <row r="37" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>72</v>
       </c>
@@ -1448,7 +1504,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="71.25">
+    <row r="38" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>74</v>
       </c>
@@ -1456,7 +1512,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="57">
+    <row r="39" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>76</v>
       </c>
@@ -1464,7 +1520,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="57">
+    <row r="40" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>78</v>
       </c>
@@ -1472,7 +1528,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="57">
+    <row r="41" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
         <v>80</v>
       </c>
@@ -1480,7 +1536,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="57">
+    <row r="42" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>82</v>
       </c>
@@ -1488,7 +1544,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="57">
+    <row r="43" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>84</v>
       </c>
@@ -1496,7 +1552,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="57">
+    <row r="44" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>86</v>
       </c>
@@ -1504,7 +1560,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="42.75">
+    <row r="45" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>88</v>
       </c>
@@ -1512,7 +1568,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="57">
+    <row r="46" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>90</v>
       </c>
@@ -1520,7 +1576,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="42.75">
+    <row r="47" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>92</v>
       </c>
@@ -1528,7 +1584,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="57">
+    <row r="48" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>94</v>
       </c>
@@ -1536,7 +1592,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="42.75">
+    <row r="49" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>96</v>
       </c>
@@ -1544,7 +1600,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="85.5">
+    <row r="50" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>98</v>
       </c>
@@ -1552,7 +1608,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="57">
+    <row r="51" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>100</v>
       </c>
@@ -1560,7 +1616,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="71.25">
+    <row r="52" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>102</v>
       </c>
@@ -1568,7 +1624,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="71.25">
+    <row r="53" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
         <v>104</v>
       </c>
@@ -1576,7 +1632,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="57">
+    <row r="54" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>106</v>
       </c>
@@ -1584,7 +1640,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="57">
+    <row r="55" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>108</v>
       </c>
@@ -1592,7 +1648,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="57">
+    <row r="56" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>110</v>
       </c>
@@ -1600,7 +1656,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="71.25">
+    <row r="57" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>112</v>
       </c>
@@ -1608,7 +1664,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="71.25">
+    <row r="58" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>114</v>
       </c>
@@ -1616,7 +1672,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="85.5">
+    <row r="59" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>116</v>
       </c>
@@ -1624,7 +1680,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="57">
+    <row r="60" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>118</v>
       </c>
@@ -1632,7 +1688,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="57">
+    <row r="61" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
         <v>120</v>
       </c>
@@ -1640,7 +1696,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="42.75">
+    <row r="62" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
         <v>122</v>
       </c>
@@ -1648,7 +1704,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="42.75">
+    <row r="63" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
         <v>124</v>
       </c>
@@ -1656,7 +1712,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="42.75">
+    <row r="64" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
         <v>126</v>
       </c>
@@ -1664,7 +1720,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="57">
+    <row r="65" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
         <v>128</v>
       </c>
@@ -1672,7 +1728,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="57">
+    <row r="66" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
         <v>130</v>
       </c>
@@ -1680,7 +1736,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="57">
+    <row r="67" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
         <v>132</v>
       </c>
@@ -1688,7 +1744,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="71.25">
+    <row r="68" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
         <v>134</v>
       </c>
@@ -1696,7 +1752,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="71.25">
+    <row r="69" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
         <v>136</v>
       </c>
@@ -1704,7 +1760,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="57">
+    <row r="70" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
         <v>138</v>
       </c>
@@ -1712,7 +1768,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="57">
+    <row r="71" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
         <v>140</v>
       </c>
@@ -1720,7 +1776,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="57">
+    <row r="72" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
         <v>142</v>
       </c>
@@ -1728,7 +1784,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="57">
+    <row r="73" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
         <v>144</v>
       </c>
@@ -1736,7 +1792,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="72" customHeight="1">
+    <row r="74" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
         <v>146</v>
       </c>
@@ -1744,7 +1800,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="71.25">
+    <row r="75" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
         <v>148</v>
       </c>
@@ -1752,7 +1808,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="71.25">
+    <row r="76" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
         <v>150</v>
       </c>
@@ -1767,18 +1823,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9CBA1D8-18C8-4CD8-9CD7-BD7764D97086}">
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25"/>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="4" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="4" customWidth="1"/>
     <col min="2" max="2" width="56" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.42578125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="32.44140625" style="6" customWidth="1"/>
     <col min="4" max="4" width="58" style="5" customWidth="1"/>
-    <col min="5" max="5" width="48.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.85546875" style="1"/>
+    <col min="5" max="5" width="48.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="42.75">
+    <row r="1" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>152</v>
       </c>
@@ -1795,7 +1851,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="69" customHeight="1">
+    <row r="2" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>157</v>
       </c>
@@ -1805,29 +1861,29 @@
       <c r="C2" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>160</v>
       </c>
       <c r="E2" s="7"/>
     </row>
-    <row r="3" spans="1:5" ht="69" customHeight="1">
+    <row r="3" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="13" t="s">
         <v>162</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="17"/>
       <c r="E3" s="7"/>
     </row>
-    <row r="4" spans="1:5" ht="107.25" customHeight="1">
+    <row r="4" spans="1:5" ht="131.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="13" t="s">
         <v>164</v>
       </c>
       <c r="C4" s="14" t="s">
@@ -1838,11 +1894,11 @@
       </c>
       <c r="E4" s="14"/>
     </row>
-    <row r="5" spans="1:5" ht="115.5" customHeight="1">
+    <row r="5" spans="1:5" ht="115.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="13" t="s">
         <v>168</v>
       </c>
       <c r="C5" s="14" t="s">
@@ -1853,11 +1909,11 @@
       </c>
       <c r="E5" s="7"/>
     </row>
-    <row r="6" spans="1:5" ht="75" customHeight="1">
+    <row r="6" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="13" t="s">
         <v>171</v>
       </c>
       <c r="C6" s="14" t="s">
@@ -1868,11 +1924,11 @@
       </c>
       <c r="E6" s="7"/>
     </row>
-    <row r="7" spans="1:5" ht="87" customHeight="1">
+    <row r="7" spans="1:5" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="13" t="s">
         <v>174</v>
       </c>
       <c r="C7" s="14" t="s">
@@ -1885,11 +1941,11 @@
         <v>176</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="95.25" customHeight="1">
+    <row r="8" spans="1:5" ht="95.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="13" t="s">
         <v>178</v>
       </c>
       <c r="C8" s="14" t="s">
@@ -1898,15 +1954,15 @@
       <c r="D8" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="16" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="75.75" customHeight="1">
+    <row r="9" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="13" t="s">
         <v>182</v>
       </c>
       <c r="C9" s="14" t="s">
@@ -1917,11 +1973,11 @@
       </c>
       <c r="E9" s="7"/>
     </row>
-    <row r="10" spans="1:5" ht="81" customHeight="1">
+    <row r="10" spans="1:5" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="13" t="s">
         <v>185</v>
       </c>
       <c r="C10" s="14" t="s">
@@ -1932,11 +1988,11 @@
       </c>
       <c r="E10" s="7"/>
     </row>
-    <row r="11" spans="1:5" ht="55.5" customHeight="1">
+    <row r="11" spans="1:5" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="13" t="s">
         <v>188</v>
       </c>
       <c r="C11" s="14" t="s">
@@ -1947,11 +2003,11 @@
       </c>
       <c r="E11" s="7"/>
     </row>
-    <row r="12" spans="1:5" ht="64.150000000000006">
+    <row r="12" spans="1:5" ht="66" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="13" t="s">
         <v>191</v>
       </c>
       <c r="C12" s="14" t="s">
@@ -1962,11 +2018,11 @@
       </c>
       <c r="E12" s="7"/>
     </row>
-    <row r="13" spans="1:5" ht="84" customHeight="1">
+    <row r="13" spans="1:5" ht="84" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="13" t="s">
         <v>194</v>
       </c>
       <c r="C13" s="14" t="s">
@@ -1977,11 +2033,11 @@
       </c>
       <c r="E13" s="7"/>
     </row>
-    <row r="14" spans="1:5" ht="84.75" customHeight="1">
+    <row r="14" spans="1:5" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="13" t="s">
         <v>197</v>
       </c>
       <c r="C14" s="14" t="s">
@@ -1992,11 +2048,11 @@
       </c>
       <c r="E14" s="7"/>
     </row>
-    <row r="15" spans="1:5" ht="76.5" customHeight="1">
+    <row r="15" spans="1:5" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="13" t="s">
         <v>200</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -2007,11 +2063,11 @@
       </c>
       <c r="E15" s="7"/>
     </row>
-    <row r="16" spans="1:5" ht="55.5" customHeight="1">
+    <row r="16" spans="1:5" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="13" t="s">
         <v>203</v>
       </c>
       <c r="C16" s="14" t="s">
@@ -2022,11 +2078,11 @@
       </c>
       <c r="E16" s="7"/>
     </row>
-    <row r="17" spans="1:5" ht="78" customHeight="1">
+    <row r="17" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="13" t="s">
         <v>206</v>
       </c>
       <c r="C17" s="14" t="s">
@@ -2036,6 +2092,92 @@
         <v>207</v>
       </c>
       <c r="E17" s="7"/>
+    </row>
+    <row r="18" spans="1:5" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
+        <v>210</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="E18" s="7"/>
+    </row>
+    <row r="19" spans="1:5" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="85.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="E20" s="7"/>
+    </row>
+    <row r="21" spans="1:5" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
+        <v>219</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>221</v>
+      </c>
+      <c r="E21" s="7"/>
+    </row>
+    <row r="22" spans="1:5" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="E22" s="7"/>
+    </row>
+    <row r="23" spans="1:5" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="E23" s="5"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B28" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2049,7 +2191,7 @@
           <x14:formula1>
             <xm:f>Valores!$A$2:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C17</xm:sqref>
+          <xm:sqref>C2:C23</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2060,24 +2202,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{632737A5-F2C7-45B2-B066-A4566BC08B73}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>165</v>
       </c>
@@ -2088,6 +2230,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010013DED8002B981F47A2AB219162B18A45" ma:contentTypeVersion="3" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="11c75646286b434d6b62b79d62284a00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="77a89e33-5ee6-4ee5-94b3-3d8acedffa3b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b189093bc8542a5f2a6028f197033518" ns2:_="">
     <xsd:import namespace="77a89e33-5ee6-4ee5-94b3-3d8acedffa3b"/>
@@ -2225,31 +2382,39 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE1E2AD2-D776-4802-A036-AA22C8535DA7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4822073-8BD3-47A0-8A52-C8DC80280AF4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5870863C-E92C-4B3F-8AED-F200998B60F2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5870863C-E92C-4B3F-8AED-F200998B60F2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4822073-8BD3-47A0-8A52-C8DC80280AF4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE1E2AD2-D776-4802-A036-AA22C8535DA7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="77a89e33-5ee6-4ee5-94b3-3d8acedffa3b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>